<commit_message>
tring to implement NSGA II
</commit_message>
<xml_diff>
--- a/tests/global_metrics.xlsx
+++ b/tests/global_metrics.xlsx
@@ -502,16 +502,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.08169</v>
+        <v>0.08517</v>
       </c>
       <c r="D2" t="n">
-        <v>0.04607</v>
+        <v>0.05448</v>
       </c>
       <c r="E2" t="n">
         <v>0.099</v>
       </c>
       <c r="F2" t="n">
-        <v>0.09702</v>
+        <v>0.10098</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -532,16 +532,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.08225</v>
+        <v>0.07803</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03779</v>
+        <v>0.03498</v>
       </c>
       <c r="E3" t="n">
         <v>0.0984</v>
       </c>
       <c r="F3" t="n">
-        <v>0.04482</v>
+        <v>0.04518</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -565,13 +565,13 @@
         <v>0.05734</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01866</v>
+        <v>0.02333</v>
       </c>
       <c r="E4" t="n">
         <v>0.1</v>
       </c>
       <c r="F4" t="n">
-        <v>0.058</v>
+        <v>0.06335</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
@@ -592,16 +592,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.07417</v>
+        <v>0.06852</v>
       </c>
       <c r="D5" t="n">
-        <v>0.02248</v>
+        <v>0.02192</v>
       </c>
       <c r="E5" t="n">
         <v>0.08989999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>0.03371</v>
+        <v>0.0309</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
@@ -626,13 +626,13 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>0.0738625</v>
+        <v>0.072265</v>
       </c>
       <c r="H6" t="n">
-        <v>0.00010117686875</v>
+        <v>0.000109138725</v>
       </c>
       <c r="I6" t="n">
-        <v>0.01005867132130283</v>
+        <v>0.01044694811894843</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -685,13 +685,13 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
-        <v>0.02083333333333333</v>
+        <v>0.02245166666666666</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0002999847222222222</v>
+        <v>0.0003653303472222222</v>
       </c>
       <c r="L8" t="n">
-        <v>0.01732006703861801</v>
+        <v>0.01911361680117665</v>
       </c>
     </row>
     <row r="9">
@@ -713,13 +713,13 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
-        <v>0.03892499999999999</v>
+        <v>0.04006833333333334</v>
       </c>
       <c r="K9" t="n">
-        <v>0.001138523858333333</v>
+        <v>0.001262232880555556</v>
       </c>
       <c r="L9" t="n">
-        <v>0.03374201917984952</v>
+        <v>0.03552791691832714</v>
       </c>
     </row>
     <row r="10">
@@ -734,16 +734,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.06832000000000001</v>
+        <v>0.06387</v>
       </c>
       <c r="D10" t="n">
-        <v>0.05545</v>
+        <v>0.05544</v>
       </c>
       <c r="E10" t="n">
         <v>0.099</v>
       </c>
       <c r="F10" t="n">
-        <v>0.09801</v>
+        <v>0.10395</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -764,16 +764,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.09068999999999999</v>
+        <v>0.08892</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0355</v>
+        <v>0.03215</v>
       </c>
       <c r="E11" t="n">
         <v>0.0984</v>
       </c>
       <c r="F11" t="n">
-        <v>0.04569</v>
+        <v>0.04499</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -794,16 +794,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.11133</v>
+        <v>0.10801</v>
       </c>
       <c r="D12" t="n">
-        <v>0.03599</v>
+        <v>0.04134</v>
       </c>
       <c r="E12" t="n">
         <v>0.1</v>
       </c>
       <c r="F12" t="n">
-        <v>0.06399000000000001</v>
+        <v>0.06533</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -824,16 +824,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.12304</v>
+        <v>0.11012</v>
       </c>
       <c r="D13" t="n">
-        <v>0.03706</v>
+        <v>0.04607</v>
       </c>
       <c r="E13" t="n">
         <v>0.08989999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>0.03482</v>
+        <v>0.02866</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
@@ -858,13 +858,13 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>0.09834499999999999</v>
+        <v>0.09272999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>0.0004346382249999999</v>
+        <v>0.00034582655</v>
       </c>
       <c r="I14" t="n">
-        <v>0.02084797891883048</v>
+        <v>0.01859641228839585</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -917,13 +917,13 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="n">
-        <v>0.02733333333333333</v>
+        <v>0.02916666666666666</v>
       </c>
       <c r="K16" t="n">
-        <v>0.0004201682555555556</v>
+        <v>0.000472414988888889</v>
       </c>
       <c r="L16" t="n">
-        <v>0.02049800613609908</v>
+        <v>0.02173510958999032</v>
       </c>
     </row>
     <row r="17">
@@ -945,13 +945,13 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="n">
-        <v>0.04041833333333333</v>
+        <v>0.04048833333333333</v>
       </c>
       <c r="K17" t="n">
-        <v>0.001199806447222222</v>
+        <v>0.001347212713888889</v>
       </c>
       <c r="L17" t="n">
-        <v>0.03463822234500816</v>
+        <v>0.03670439638366076</v>
       </c>
     </row>
   </sheetData>

</xml_diff>